<commit_message>
chore: update match data [scraper]
</commit_message>
<xml_diff>
--- a/futbolaragon_data.xlsx
+++ b/futbolaragon_data.xlsx
@@ -2528,7 +2528,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -2780,7 +2780,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -4859,7 +4859,7 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
@@ -5930,7 +5930,7 @@
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -7694,7 +7694,7 @@
         <v>0</v>
       </c>
       <c r="L88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
         <v>0</v>
       </c>
       <c r="L96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M96" t="inlineStr">
         <is>
@@ -10088,7 +10088,7 @@
         <v>0</v>
       </c>
       <c r="L126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -10151,7 +10151,7 @@
         <v>0</v>
       </c>
       <c r="L127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M127" t="inlineStr">
         <is>
@@ -10340,7 +10340,7 @@
         <v>0</v>
       </c>
       <c r="L130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
         <v>0</v>
       </c>
       <c r="L135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -11222,7 +11222,7 @@
         <v>0</v>
       </c>
       <c r="L144" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M144" t="inlineStr">
         <is>
@@ -11285,7 +11285,7 @@
         <v>0</v>
       </c>
       <c r="L145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M145" t="inlineStr">
         <is>
@@ -11411,7 +11411,7 @@
         <v>0</v>
       </c>
       <c r="L147" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -11474,7 +11474,7 @@
         <v>0</v>
       </c>
       <c r="L148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -12041,7 +12041,7 @@
         <v>0</v>
       </c>
       <c r="L157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -12293,7 +12293,7 @@
         <v>0</v>
       </c>
       <c r="L161" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M161" t="inlineStr">
         <is>
@@ -12419,7 +12419,7 @@
         <v>0</v>
       </c>
       <c r="L163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -13112,7 +13112,7 @@
         <v>0</v>
       </c>
       <c r="L174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -13931,7 +13931,7 @@
         <v>0</v>
       </c>
       <c r="L187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -14246,7 +14246,7 @@
         <v>0</v>
       </c>
       <c r="L192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M192" t="inlineStr">
         <is>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="L203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M203" t="inlineStr">
         <is>
@@ -15380,7 +15380,7 @@
         <v>0</v>
       </c>
       <c r="L210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
@@ -15506,7 +15506,7 @@
         <v>0</v>
       </c>
       <c r="L212" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
@@ -15569,7 +15569,7 @@
         <v>0</v>
       </c>
       <c r="L213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M213" t="inlineStr">
         <is>
@@ -15758,7 +15758,7 @@
         <v>0</v>
       </c>
       <c r="L216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M216" t="inlineStr">
         <is>
@@ -15821,7 +15821,7 @@
         <v>0</v>
       </c>
       <c r="L217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M217" t="inlineStr">
         <is>
@@ -16010,7 +16010,7 @@
         <v>0</v>
       </c>
       <c r="L220" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
@@ -16388,7 +16388,7 @@
         <v>0</v>
       </c>
       <c r="L226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M226" t="inlineStr">
         <is>
@@ -17018,7 +17018,7 @@
         <v>0</v>
       </c>
       <c r="L236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -18656,7 +18656,7 @@
         <v>0</v>
       </c>
       <c r="L262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -20546,7 +20546,7 @@
         <v>0</v>
       </c>
       <c r="L292" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -21239,7 +21239,7 @@
         <v>0</v>
       </c>
       <c r="L303" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -23633,7 +23633,7 @@
         <v>0</v>
       </c>
       <c r="L341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M341" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
         <v>0</v>
       </c>
       <c r="L343" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M343" t="inlineStr">
         <is>
@@ -26342,7 +26342,7 @@
         <v>0</v>
       </c>
       <c r="L384" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M384" t="inlineStr">
         <is>
@@ -26909,7 +26909,7 @@
         <v>0</v>
       </c>
       <c r="L393" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M393" t="inlineStr">
         <is>
@@ -27161,7 +27161,7 @@
         <v>0</v>
       </c>
       <c r="L397" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M397" t="inlineStr">
         <is>
@@ -27539,7 +27539,7 @@
         <v>0</v>
       </c>
       <c r="L403" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M403" t="inlineStr">
         <is>
@@ -27602,7 +27602,7 @@
         <v>0</v>
       </c>
       <c r="L404" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M404" t="inlineStr">
         <is>
@@ -27665,7 +27665,7 @@
         <v>0</v>
       </c>
       <c r="L405" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M405" t="inlineStr">
         <is>
@@ -28736,7 +28736,7 @@
         <v>0</v>
       </c>
       <c r="L422" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M422" t="inlineStr">
         <is>
@@ -28925,7 +28925,7 @@
         <v>0</v>
       </c>
       <c r="L425" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M425" t="inlineStr">
         <is>
@@ -29177,7 +29177,7 @@
         <v>0</v>
       </c>
       <c r="L429" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M429" t="inlineStr">
         <is>
@@ -30815,7 +30815,7 @@
         <v>0</v>
       </c>
       <c r="L455" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M455" t="inlineStr">
         <is>
@@ -30878,7 +30878,7 @@
         <v>0</v>
       </c>
       <c r="L456" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M456" t="inlineStr">
         <is>
@@ -31571,7 +31571,7 @@
         <v>0</v>
       </c>
       <c r="L467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M467" t="inlineStr">
         <is>
@@ -31886,7 +31886,7 @@
         <v>0</v>
       </c>
       <c r="L472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M472" t="inlineStr">
         <is>
@@ -32075,7 +32075,7 @@
         <v>0</v>
       </c>
       <c r="L475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M475" t="inlineStr">
         <is>
@@ -33713,7 +33713,7 @@
         <v>0</v>
       </c>
       <c r="L501" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M501" t="inlineStr">
         <is>
@@ -34658,7 +34658,7 @@
         <v>0</v>
       </c>
       <c r="L516" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M516" t="inlineStr">
         <is>
@@ -35036,7 +35036,7 @@
         <v>0</v>
       </c>
       <c r="L522" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M522" t="inlineStr">
         <is>
@@ -35729,7 +35729,7 @@
         <v>0</v>
       </c>
       <c r="L533" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M533" t="inlineStr">
         <is>
@@ -36107,7 +36107,7 @@
         <v>0</v>
       </c>
       <c r="L539" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M539" t="inlineStr">
         <is>
@@ -36737,7 +36737,7 @@
         <v>0</v>
       </c>
       <c r="L549" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M549" t="inlineStr">
         <is>
@@ -37745,7 +37745,7 @@
         <v>0</v>
       </c>
       <c r="L565" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M565" t="inlineStr">
         <is>
@@ -38375,7 +38375,7 @@
         <v>0</v>
       </c>
       <c r="L575" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M575" t="inlineStr">
         <is>
@@ -39005,7 +39005,7 @@
         <v>0</v>
       </c>
       <c r="L585" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M585" t="inlineStr">
         <is>
@@ -39131,7 +39131,7 @@
         <v>0</v>
       </c>
       <c r="L587" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M587" t="inlineStr">
         <is>
@@ -39383,7 +39383,7 @@
         <v>0</v>
       </c>
       <c r="L591" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M591" t="inlineStr">
         <is>
@@ -40076,7 +40076,7 @@
         <v>0</v>
       </c>
       <c r="L602" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M602" t="inlineStr">
         <is>
@@ -40643,7 +40643,7 @@
         <v>0</v>
       </c>
       <c r="L611" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M611" t="inlineStr">
         <is>
@@ -41210,7 +41210,7 @@
         <v>0</v>
       </c>
       <c r="L620" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M620" t="inlineStr">
         <is>
@@ -41714,7 +41714,7 @@
         <v>0</v>
       </c>
       <c r="L628" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M628" t="inlineStr">
         <is>
@@ -42533,7 +42533,7 @@
         <v>0</v>
       </c>
       <c r="L641" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M641" t="inlineStr">
         <is>
@@ -44108,7 +44108,7 @@
         <v>0</v>
       </c>
       <c r="L666" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M666" t="inlineStr">
         <is>
@@ -45242,7 +45242,7 @@
         <v>0</v>
       </c>
       <c r="L684" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M684" t="inlineStr">
         <is>
@@ -47636,7 +47636,7 @@
         <v>0</v>
       </c>
       <c r="L722" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M722" t="inlineStr">
         <is>
@@ -49022,7 +49022,7 @@
         <v>0</v>
       </c>
       <c r="L744" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M744" t="inlineStr">
         <is>
@@ -49148,7 +49148,7 @@
         <v>0</v>
       </c>
       <c r="L746" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M746" t="inlineStr">
         <is>
@@ -49967,7 +49967,7 @@
         <v>0</v>
       </c>
       <c r="L759" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M759" t="inlineStr">
         <is>
@@ -50282,7 +50282,7 @@
         <v>0</v>
       </c>
       <c r="L764" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M764" t="inlineStr">
         <is>
@@ -55133,7 +55133,7 @@
         <v>0</v>
       </c>
       <c r="L841" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M841" t="inlineStr">
         <is>
@@ -55574,7 +55574,7 @@
         <v>0</v>
       </c>
       <c r="L848" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M848" t="inlineStr">
         <is>
@@ -55889,7 +55889,7 @@
         <v>0</v>
       </c>
       <c r="L853" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M853" t="inlineStr">
         <is>
@@ -55952,7 +55952,7 @@
         <v>0</v>
       </c>
       <c r="L854" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M854" t="inlineStr">
         <is>
@@ -56393,7 +56393,7 @@
         <v>0</v>
       </c>
       <c r="L861" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M861" t="inlineStr">
         <is>
@@ -56582,7 +56582,7 @@
         <v>0</v>
       </c>
       <c r="L864" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M864" t="inlineStr">
         <is>
@@ -56708,7 +56708,7 @@
         <v>0</v>
       </c>
       <c r="L866" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M866" t="inlineStr">
         <is>
@@ -57023,7 +57023,7 @@
         <v>0</v>
       </c>
       <c r="L871" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M871" t="inlineStr">
         <is>
@@ -57272,7 +57272,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -57309,7 +57309,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -57383,7 +57383,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -57420,7 +57420,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
@@ -57457,7 +57457,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
@@ -57494,7 +57494,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -57531,7 +57531,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
@@ -57568,7 +57568,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
@@ -57605,7 +57605,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
@@ -57642,7 +57642,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H12" t="n">
         <v>9</v>
@@ -57679,7 +57679,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -57716,7 +57716,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -57753,7 +57753,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H15" t="n">
         <v>6</v>
@@ -57864,7 +57864,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18" t="n">
         <v>6</v>
@@ -57938,7 +57938,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
         <v>3</v>
@@ -57975,7 +57975,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>9</v>
@@ -58012,7 +58012,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H22" t="n">
         <v>5</v>
@@ -58086,7 +58086,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -58160,7 +58160,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
         <v>13</v>
@@ -58197,7 +58197,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H27" t="n">
         <v>9</v>
@@ -58271,7 +58271,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
         <v>6</v>
@@ -58345,7 +58345,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
         <v>10</v>
@@ -58382,7 +58382,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>10</v>
@@ -58419,7 +58419,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
         <v>6</v>
@@ -58456,7 +58456,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H34" t="n">
         <v>8</v>
@@ -58567,7 +58567,7 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H37" t="n">
         <v>10</v>
@@ -58604,7 +58604,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -58641,7 +58641,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H39" t="n">
         <v>2</v>
@@ -58678,7 +58678,7 @@
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40" t="n">
         <v>7</v>
@@ -59085,7 +59085,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H51" t="n">
         <v>4</v>
@@ -59122,7 +59122,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
refactor: improve card parsing logic and enhance fuzzy matching for player stats in futbolaragon_scraper.py
</commit_message>
<xml_diff>
--- a/futbolaragon_data.xlsx
+++ b/futbolaragon_data.xlsx
@@ -10,13 +10,11 @@
     <sheet name="Detalle Partidos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Datos Jugadores" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Resumen Plantilla" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="LOUREDA ALVAREZ, JAIME" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detalle Partidos'!$A$1:$H$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos Jugadores'!$A$1:$O$873</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumen Plantilla'!$A$1:$K$62</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'LOUREDA ALVAREZ, JAIME'!$A$1:$O$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2528,7 +2526,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -2591,7 +2589,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -2780,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -3536,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -4859,7 +4857,7 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
@@ -5930,7 +5928,7 @@
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -7694,7 +7692,7 @@
         <v>0</v>
       </c>
       <c r="L88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8198,7 +8196,7 @@
         <v>0</v>
       </c>
       <c r="L96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M96" t="inlineStr">
         <is>
@@ -10088,7 +10086,7 @@
         <v>0</v>
       </c>
       <c r="L126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -10151,7 +10149,7 @@
         <v>0</v>
       </c>
       <c r="L127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M127" t="inlineStr">
         <is>
@@ -10340,7 +10338,7 @@
         <v>0</v>
       </c>
       <c r="L130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -10655,7 +10653,7 @@
         <v>0</v>
       </c>
       <c r="L135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -11222,7 +11220,7 @@
         <v>0</v>
       </c>
       <c r="L144" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M144" t="inlineStr">
         <is>
@@ -11285,7 +11283,7 @@
         <v>0</v>
       </c>
       <c r="L145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M145" t="inlineStr">
         <is>
@@ -11411,7 +11409,7 @@
         <v>0</v>
       </c>
       <c r="L147" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -11474,7 +11472,7 @@
         <v>0</v>
       </c>
       <c r="L148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -12041,7 +12039,7 @@
         <v>0</v>
       </c>
       <c r="L157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -12293,7 +12291,7 @@
         <v>0</v>
       </c>
       <c r="L161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M161" t="inlineStr">
         <is>
@@ -12419,7 +12417,7 @@
         <v>0</v>
       </c>
       <c r="L163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -13112,7 +13110,7 @@
         <v>0</v>
       </c>
       <c r="L174" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -13931,7 +13929,7 @@
         <v>0</v>
       </c>
       <c r="L187" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -14246,7 +14244,7 @@
         <v>0</v>
       </c>
       <c r="L192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M192" t="inlineStr">
         <is>
@@ -14939,7 +14937,7 @@
         <v>0</v>
       </c>
       <c r="L203" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M203" t="inlineStr">
         <is>
@@ -15380,7 +15378,7 @@
         <v>0</v>
       </c>
       <c r="L210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
@@ -15506,7 +15504,7 @@
         <v>0</v>
       </c>
       <c r="L212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
@@ -15569,7 +15567,7 @@
         <v>0</v>
       </c>
       <c r="L213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M213" t="inlineStr">
         <is>
@@ -15758,7 +15756,7 @@
         <v>0</v>
       </c>
       <c r="L216" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M216" t="inlineStr">
         <is>
@@ -15821,7 +15819,7 @@
         <v>0</v>
       </c>
       <c r="L217" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M217" t="inlineStr">
         <is>
@@ -16010,7 +16008,7 @@
         <v>0</v>
       </c>
       <c r="L220" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
@@ -16388,7 +16386,7 @@
         <v>0</v>
       </c>
       <c r="L226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M226" t="inlineStr">
         <is>
@@ -17018,7 +17016,7 @@
         <v>0</v>
       </c>
       <c r="L236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -18656,7 +18654,7 @@
         <v>0</v>
       </c>
       <c r="L262" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -20546,7 +20544,7 @@
         <v>0</v>
       </c>
       <c r="L292" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -20924,7 +20922,7 @@
         <v>0</v>
       </c>
       <c r="L298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -21239,7 +21237,7 @@
         <v>0</v>
       </c>
       <c r="L303" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -23381,7 +23379,7 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -23444,7 +23442,7 @@
         <v>0</v>
       </c>
       <c r="L338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M338" t="inlineStr">
         <is>
@@ -23633,7 +23631,7 @@
         <v>0</v>
       </c>
       <c r="L341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M341" t="inlineStr">
         <is>
@@ -23759,7 +23757,7 @@
         <v>0</v>
       </c>
       <c r="L343" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M343" t="inlineStr">
         <is>
@@ -26342,7 +26340,7 @@
         <v>0</v>
       </c>
       <c r="L384" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M384" t="inlineStr">
         <is>
@@ -26909,7 +26907,7 @@
         <v>0</v>
       </c>
       <c r="L393" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M393" t="inlineStr">
         <is>
@@ -27161,7 +27159,7 @@
         <v>0</v>
       </c>
       <c r="L397" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M397" t="inlineStr">
         <is>
@@ -27539,7 +27537,7 @@
         <v>0</v>
       </c>
       <c r="L403" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M403" t="inlineStr">
         <is>
@@ -27602,7 +27600,7 @@
         <v>0</v>
       </c>
       <c r="L404" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M404" t="inlineStr">
         <is>
@@ -27665,7 +27663,7 @@
         <v>0</v>
       </c>
       <c r="L405" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M405" t="inlineStr">
         <is>
@@ -28736,7 +28734,7 @@
         <v>0</v>
       </c>
       <c r="L422" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M422" t="inlineStr">
         <is>
@@ -28925,7 +28923,7 @@
         <v>0</v>
       </c>
       <c r="L425" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M425" t="inlineStr">
         <is>
@@ -29177,7 +29175,7 @@
         <v>0</v>
       </c>
       <c r="L429" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M429" t="inlineStr">
         <is>
@@ -30815,7 +30813,7 @@
         <v>0</v>
       </c>
       <c r="L455" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M455" t="inlineStr">
         <is>
@@ -30878,7 +30876,7 @@
         <v>0</v>
       </c>
       <c r="L456" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M456" t="inlineStr">
         <is>
@@ -31571,7 +31569,7 @@
         <v>0</v>
       </c>
       <c r="L467" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M467" t="inlineStr">
         <is>
@@ -31886,7 +31884,7 @@
         <v>0</v>
       </c>
       <c r="L472" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M472" t="inlineStr">
         <is>
@@ -32075,7 +32073,7 @@
         <v>0</v>
       </c>
       <c r="L475" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M475" t="inlineStr">
         <is>
@@ -33713,7 +33711,7 @@
         <v>0</v>
       </c>
       <c r="L501" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M501" t="inlineStr">
         <is>
@@ -34658,7 +34656,7 @@
         <v>0</v>
       </c>
       <c r="L516" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M516" t="inlineStr">
         <is>
@@ -35036,7 +35034,7 @@
         <v>0</v>
       </c>
       <c r="L522" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M522" t="inlineStr">
         <is>
@@ -35729,7 +35727,7 @@
         <v>0</v>
       </c>
       <c r="L533" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M533" t="inlineStr">
         <is>
@@ -35918,7 +35916,7 @@
         <v>0</v>
       </c>
       <c r="L536" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M536" t="inlineStr">
         <is>
@@ -36107,7 +36105,7 @@
         <v>0</v>
       </c>
       <c r="L539" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M539" t="inlineStr">
         <is>
@@ -36737,7 +36735,7 @@
         <v>0</v>
       </c>
       <c r="L549" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M549" t="inlineStr">
         <is>
@@ -37745,7 +37743,7 @@
         <v>0</v>
       </c>
       <c r="L565" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M565" t="inlineStr">
         <is>
@@ -38375,7 +38373,7 @@
         <v>0</v>
       </c>
       <c r="L575" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M575" t="inlineStr">
         <is>
@@ -39005,7 +39003,7 @@
         <v>0</v>
       </c>
       <c r="L585" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M585" t="inlineStr">
         <is>
@@ -39131,7 +39129,7 @@
         <v>0</v>
       </c>
       <c r="L587" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M587" t="inlineStr">
         <is>
@@ -39383,7 +39381,7 @@
         <v>0</v>
       </c>
       <c r="L591" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M591" t="inlineStr">
         <is>
@@ -40076,7 +40074,7 @@
         <v>0</v>
       </c>
       <c r="L602" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M602" t="inlineStr">
         <is>
@@ -40643,7 +40641,7 @@
         <v>0</v>
       </c>
       <c r="L611" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M611" t="inlineStr">
         <is>
@@ -41210,7 +41208,7 @@
         <v>0</v>
       </c>
       <c r="L620" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M620" t="inlineStr">
         <is>
@@ -41714,7 +41712,7 @@
         <v>0</v>
       </c>
       <c r="L628" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M628" t="inlineStr">
         <is>
@@ -42533,7 +42531,7 @@
         <v>0</v>
       </c>
       <c r="L641" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M641" t="inlineStr">
         <is>
@@ -44108,7 +44106,7 @@
         <v>0</v>
       </c>
       <c r="L666" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M666" t="inlineStr">
         <is>
@@ -45242,7 +45240,7 @@
         <v>0</v>
       </c>
       <c r="L684" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M684" t="inlineStr">
         <is>
@@ -47636,7 +47634,7 @@
         <v>0</v>
       </c>
       <c r="L722" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M722" t="inlineStr">
         <is>
@@ -49022,7 +49020,7 @@
         <v>0</v>
       </c>
       <c r="L744" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M744" t="inlineStr">
         <is>
@@ -49148,7 +49146,7 @@
         <v>0</v>
       </c>
       <c r="L746" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M746" t="inlineStr">
         <is>
@@ -49967,7 +49965,7 @@
         <v>0</v>
       </c>
       <c r="L759" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M759" t="inlineStr">
         <is>
@@ -50282,7 +50280,7 @@
         <v>0</v>
       </c>
       <c r="L764" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M764" t="inlineStr">
         <is>
@@ -55133,7 +55131,7 @@
         <v>0</v>
       </c>
       <c r="L841" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M841" t="inlineStr">
         <is>
@@ -55574,7 +55572,7 @@
         <v>0</v>
       </c>
       <c r="L848" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M848" t="inlineStr">
         <is>
@@ -55889,7 +55887,7 @@
         <v>0</v>
       </c>
       <c r="L853" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M853" t="inlineStr">
         <is>
@@ -55952,7 +55950,7 @@
         <v>0</v>
       </c>
       <c r="L854" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M854" t="inlineStr">
         <is>
@@ -56393,7 +56391,7 @@
         <v>0</v>
       </c>
       <c r="L861" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M861" t="inlineStr">
         <is>
@@ -56582,7 +56580,7 @@
         <v>0</v>
       </c>
       <c r="L864" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M864" t="inlineStr">
         <is>
@@ -56708,7 +56706,7 @@
         <v>0</v>
       </c>
       <c r="L866" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M866" t="inlineStr">
         <is>
@@ -57023,7 +57021,7 @@
         <v>0</v>
       </c>
       <c r="L871" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M871" t="inlineStr">
         <is>
@@ -57272,7 +57270,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -57309,7 +57307,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -57383,7 +57381,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -57420,7 +57418,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
@@ -57457,7 +57455,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
@@ -57494,7 +57492,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -57531,7 +57529,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
@@ -57568,7 +57566,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
@@ -57605,7 +57603,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
@@ -57642,7 +57640,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>9</v>
@@ -57679,7 +57677,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -57716,7 +57714,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -57753,7 +57751,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>6</v>
@@ -57864,7 +57862,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
         <v>6</v>
@@ -57938,7 +57936,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>3</v>
@@ -57975,7 +57973,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>9</v>
@@ -58012,7 +58010,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
         <v>5</v>
@@ -58086,7 +58084,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -58160,7 +58158,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
         <v>13</v>
@@ -58197,7 +58195,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
         <v>9</v>
@@ -58271,7 +58269,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
         <v>6</v>
@@ -58345,7 +58343,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
         <v>10</v>
@@ -58382,7 +58380,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>10</v>
@@ -58419,7 +58417,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>6</v>
@@ -58456,7 +58454,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
         <v>8</v>
@@ -58530,7 +58528,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -58567,7 +58565,7 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
         <v>10</v>
@@ -58604,7 +58602,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -58641,7 +58639,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
         <v>2</v>
@@ -58678,7 +58676,7 @@
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>7</v>
@@ -59085,7 +59083,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H51" t="n">
         <v>4</v>
@@ -59122,7 +59120,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H52" t="n">
         <v>3</v>
@@ -59511,1562 +59509,4 @@
   <autoFilter ref="A1:K62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Partido</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Rival</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Condición</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Jugador</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Dorsal</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Titular</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Min. Entrada</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Min. Salida</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Minutos Jugados</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Goles</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Amarillas</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Rojas</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Jugó</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Suplente Usado</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Titularidad_num</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>STADIUM CASABLANCA-C.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>STADIUM CASABLANCA-C.D.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I2" t="n">
-        <v>20</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs SAN AGUSTIN-C.D.</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SAN AGUSTIN-C.D.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>51</v>
-      </c>
-      <c r="H3" t="n">
-        <v>80</v>
-      </c>
-      <c r="I3" t="n">
-        <v>29</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BINEFAR-FUTBOL BASE vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BINEFAR-FUTBOL BASE</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>80</v>
-      </c>
-      <c r="I4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs MONZÓN FÚTBOL BASE - AT. AHP Guarvi</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MONZÓN FÚTBOL BASE - AT. AHP Guarvi</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>57</v>
-      </c>
-      <c r="H5" t="n">
-        <v>80</v>
-      </c>
-      <c r="I5" t="n">
-        <v>23</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MONTECARLO-U.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MONTECARLO-U.D.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>61</v>
-      </c>
-      <c r="H6" t="n">
-        <v>80</v>
-      </c>
-      <c r="I6" t="n">
-        <v>19</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs REAL ZARAGOZA S.A.D.</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>REAL ZARAGOZA S.A.D.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>58</v>
-      </c>
-      <c r="H7" t="n">
-        <v>80</v>
-      </c>
-      <c r="I7" t="n">
-        <v>22</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs ESTADIO MIRALBUENO EL OLIVAR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ESTADIO MIRALBUENO EL OLIVAR</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>80</v>
-      </c>
-      <c r="I8" t="n">
-        <v>80</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>OLIVER-C.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>OLIVER-C.D.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>55</v>
-      </c>
-      <c r="I9" t="n">
-        <v>55</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs HUESCA-S.D. ESCUELA DE FUTBOL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. ESCUELA DE FUTBOL</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>46</v>
-      </c>
-      <c r="H10" t="n">
-        <v>80</v>
-      </c>
-      <c r="I10" t="n">
-        <v>34</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FRAGA-FÚTBOL BASE vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>FRAGA-FÚTBOL BASE</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>54</v>
-      </c>
-      <c r="H11" t="n">
-        <v>80</v>
-      </c>
-      <c r="I11" t="n">
-        <v>26</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs CALATAYUD-EFB</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CALATAYUD-EFB</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>41</v>
-      </c>
-      <c r="H12" t="n">
-        <v>80</v>
-      </c>
-      <c r="I12" t="n">
-        <v>39</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs HERNAN CORTES JUNQUERA-C.F.</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HERNAN CORTES JUNQUERA-C.F.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>63</v>
-      </c>
-      <c r="I13" t="n">
-        <v>63</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CUARTE-C.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CUARTE-C.D.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>80</v>
-      </c>
-      <c r="I14" t="n">
-        <v>80</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs RACING CLUB ZARAGOZA</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RACING CLUB ZARAGOZA</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>74</v>
-      </c>
-      <c r="H15" t="n">
-        <v>80</v>
-      </c>
-      <c r="I15" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs STADIUM CASABLANCA-C.D.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>STADIUM CASABLANCA-C.D.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>63</v>
-      </c>
-      <c r="H16" t="n">
-        <v>80</v>
-      </c>
-      <c r="I16" t="n">
-        <v>17</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SAN AGUSTIN-C.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SAN AGUSTIN-C.D.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>54</v>
-      </c>
-      <c r="H17" t="n">
-        <v>80</v>
-      </c>
-      <c r="I17" t="n">
-        <v>26</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs BINEFAR-FUTBOL BASE</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>BINEFAR-FUTBOL BASE</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>80</v>
-      </c>
-      <c r="I18" t="n">
-        <v>80</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MONZÓN FÚTBOL BASE - AT. AHP Guarvi vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>MONZÓN FÚTBOL BASE - AT. AHP Guarvi</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>80</v>
-      </c>
-      <c r="I19" t="n">
-        <v>80</v>
-      </c>
-      <c r="J19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs MONTECARLO-U.D.</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>MONTECARLO-U.D.</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>53</v>
-      </c>
-      <c r="H20" t="n">
-        <v>80</v>
-      </c>
-      <c r="I20" t="n">
-        <v>27</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>REAL ZARAGOZA S.A.D. vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>REAL ZARAGOZA S.A.D.</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>66</v>
-      </c>
-      <c r="H21" t="n">
-        <v>80</v>
-      </c>
-      <c r="I21" t="n">
-        <v>14</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs BALSAS PICARRAL-U.D.</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BALSAS PICARRAL-U.D.</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>80</v>
-      </c>
-      <c r="I22" t="n">
-        <v>80</v>
-      </c>
-      <c r="J22" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ESTADIO MIRALBUENO EL OLIVAR vs HUESCA-S.D.</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>ESTADIO MIRALBUENO EL OLIVAR</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Visitante</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H23" t="n">
-        <v>80</v>
-      </c>
-      <c r="I23" t="n">
-        <v>40</v>
-      </c>
-      <c r="J23" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>HUESCA-S.D. vs OLIVER-C.D.</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>OLIVER-C.D.</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>LOUREDA ALVAREZ, JAIME</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:O24"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>